<commit_message>
Explore Pants: unidades a producir por proporción compra color/talla
- Ancla 2.908 und al 80% pendiente; color según % del pedido (no kg→und)
- Género/talla desde ventas con boost KIDS +12%; excluye talla 1
- Consumo tela referencial: CAB 0.30, DAMA 0.25, KIDS 0.22 kg/und
- Excel enfocado en producción; hoja tela como referencia del pedido ya hecho

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/EXPLORE_PANTS_Proyeccion_Produccion.xlsx
+++ b/EXPLORE_PANTS_Proyeccion_Produccion.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Resumen" sheetId="1" r:id="rId1"/>
     <sheet name="Cantidades por Colores" sheetId="2" r:id="rId2"/>
     <sheet name="Producción por Talla" sheetId="3" r:id="rId3"/>
-    <sheet name="Compra de Tela" sheetId="4" r:id="rId4"/>
+    <sheet name="Tela Comprada (ref.)" sheetId="4" r:id="rId4"/>
     <sheet name="Compra en 2 Órdenes" sheetId="5" r:id="rId5"/>
     <sheet name="Producción Color × Talla" sheetId="6" r:id="rId6"/>
     <sheet name="Metodología" sheetId="7" r:id="rId7"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="105">
   <si>
     <t>EXPLORE PANTS — PROYECCIÓN ANCLADA A JUSTIFICACIÓN NOVAKTEX</t>
   </si>
@@ -40,16 +40,22 @@
     <t>Stock actual dashboard: 3,249 und</t>
   </si>
   <si>
-    <t>Tela Explore (kg con 20% merma): 1089 kg</t>
+    <t>Tela ya comprada (referencia): 1089 kg Explore</t>
   </si>
   <si>
     <t>Pedido total archivo (Explore + Shorts): 1088 kg · split 65% / 35%</t>
   </si>
   <si>
-    <t>Distribución color×talla/género: proporcional a ventas del dashboard</t>
-  </si>
-  <si>
-    <t>Gris (ventas) → Gris Oscuro (producción/tela)</t>
+    <t>Color: proporción del pedido (Negro 38% · Gris Oscuro 33% · Kaki 14% · Azul 8% · Verde 6%)</t>
+  </si>
+  <si>
+    <t>Talla/género: curva de ventas del dashboard · KIDS con boost moderado (+12%)</t>
+  </si>
+  <si>
+    <t>Consumo referencial: CAB 0.3 · DAMA 0.25 · KIDS 0.22 kg/und</t>
+  </si>
+  <si>
+    <t>Gris (ventas) → Gris Oscuro (producción)</t>
   </si>
   <si>
     <t>Demanda mensual (justificación)</t>
@@ -112,7 +118,7 @@
     <t>TOTAL</t>
   </si>
   <si>
-    <t>EXPLORE PANTS — CANTIDADES POR COLOR (meta = kg justificación)</t>
+    <t>EXPLORE PANTS — UNIDADES A PRODUCIR POR COLOR</t>
   </si>
   <si>
     <t>Color</t>
@@ -121,13 +127,13 @@
     <t>Und a producir</t>
   </si>
   <si>
-    <t>% del total</t>
-  </si>
-  <si>
-    <t>Kg tela (justif.)</t>
-  </si>
-  <si>
-    <t>Kg consumo neto</t>
+    <t>% compra (color)</t>
+  </si>
+  <si>
+    <t>Kg tela comprada (ref.)</t>
+  </si>
+  <si>
+    <t>Kg neto (ref.)</t>
   </si>
   <si>
     <t>Negro</t>
@@ -208,21 +214,30 @@
     <t>12</t>
   </si>
   <si>
-    <t>EXPLORE PANTS — COMPRA TELA NOVAKTEX REPEL</t>
-  </si>
-  <si>
-    <t>Und</t>
+    <t>EXPLORE PANTS — TELA NOVAKTEX REPEL YA COMPRADA</t>
+  </si>
+  <si>
+    <t>La tela ya está pedida. Esta hoja es referencia del pedido, no recalcula las und.</t>
+  </si>
+  <si>
+    <t>% color compra</t>
   </si>
   <si>
     <t>Kg compra (+20% SS)</t>
   </si>
   <si>
-    <t>Consumo kg/und implícito</t>
+    <t>Kg neto</t>
   </si>
   <si>
     <t>TOTAL EXPLORE</t>
   </si>
   <si>
+    <t>Consumo referencial por género (kg/und)</t>
+  </si>
+  <si>
+    <t>Consumo ref.</t>
+  </si>
+  <si>
     <t>PROPUESTA COMPRA 65% AHORA / 35% SEPTIEMBRE (archivo justificación)</t>
   </si>
   <si>
@@ -301,19 +316,25 @@
     <t>METODOLOGÍA — EXPLORE PANTS</t>
   </si>
   <si>
-    <t>1. La cantidad TOTAL a producir (2,908 und) viene del 80% pendiente en la justificación Novaktex.</t>
-  </si>
-  <si>
-    <t>2. El reparto por COLOR sigue el peso de kg de tela del archivo: Negro 414 · Gris Oscuro 361 · Kaki 157 · Azul 91 · Verde 66 kg.</t>
-  </si>
-  <si>
-    <t>3. Dentro de cada color, género y talla se reparten según ventas del dashboard Explore Pants.</t>
-  </si>
-  <si>
-    <t>4. La demanda Jul–Dic (2,228 und) y escenarios mensuales se mantienen del archivo de justificación.</t>
-  </si>
-  <si>
-    <t>5. Compra de tela en 2 órdenes (65%/35%) es réplica del pedido aprobado; Shorts R1 van en la misma orden pero son producto aparte.</t>
+    <t>1. TOTAL a producir: 2,908 und (80% pendiente, justificación Novaktex). La tela ya está comprada.</t>
+  </si>
+  <si>
+    <t>2. COLOR: proporción del pedido de tela — Negro 38.0% · Gris Oscuro 33.1% · Kaki 14.4% · Azul Marino 8.4% · Verde Militar 6.1%.</t>
+  </si>
+  <si>
+    <t>3. GÉNERO y TALLA: curva de ventas del dashboard dentro de cada color; KIDS con boost +12% sobre su share de ventas.</t>
+  </si>
+  <si>
+    <t>4. Consumo referencial (no define und): CAB 0.3 · DAMA 0.25 · KIDS 0.22 kg/und.</t>
+  </si>
+  <si>
+    <t>5. KIDS excluye talla 1 en producción (venta marginal). Gris (ventas) → Gris Oscuro (producción).</t>
+  </si>
+  <si>
+    <t>6. Demanda Jul–Dic (2,228 und) y escenarios mensuales del archivo de justificación.</t>
+  </si>
+  <si>
+    <t>7. Hoja 'Compra en 2 Órdenes': réplica del pedido de tela aprobado (referencia logística).</t>
   </si>
 </sst>
 </file>
@@ -712,7 +733,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="48.7109375" customWidth="1"/>
@@ -772,33 +793,27 @@
         <v>9</v>
       </c>
     </row>
+    <row r="12" spans="1:4">
+      <c r="A12" t="s">
+        <v>10</v>
+      </c>
+    </row>
     <row r="13" spans="1:4">
-      <c r="A13" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="3" t="s">
+      <c r="A13" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="3" t="s">
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
-      <c r="A15" t="s">
+    <row r="16" spans="1:4">
+      <c r="A16" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="4">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" t="s">
+      <c r="B16" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="B16" s="4">
-        <v>261</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -806,7 +821,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="4">
-        <v>308</v>
+        <v>42</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -814,7 +829,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="4">
-        <v>421</v>
+        <v>261</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -822,7 +837,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="4">
-        <v>598</v>
+        <v>308</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -830,75 +845,69 @@
         <v>18</v>
       </c>
       <c r="B20" s="4">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="4">
         <v>598</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
-      <c r="A21" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B21" s="4">
+    <row r="22" spans="1:3">
+      <c r="A22" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="4">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" s="4">
         <v>2228</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
-      <c r="A23" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3">
-      <c r="A24" t="s">
-        <v>21</v>
-      </c>
-      <c r="B24" s="4">
+    <row r="25" spans="1:3">
+      <c r="A25" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" t="s">
+        <v>23</v>
+      </c>
+      <c r="B26" s="4">
         <v>760</v>
       </c>
-      <c r="C24" s="4">
+      <c r="C26" s="4">
         <v>1021</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
-      <c r="A25" t="s">
-        <v>22</v>
-      </c>
-      <c r="B25" s="4">
+    <row r="27" spans="1:3">
+      <c r="A27" t="s">
+        <v>24</v>
+      </c>
+      <c r="B27" s="4">
         <v>3668</v>
       </c>
-      <c r="C25" s="4">
+      <c r="C27" s="4">
         <v>3929</v>
       </c>
     </row>
-    <row r="27" spans="1:3">
-      <c r="A27" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C27" s="3" t="s">
+    <row r="29" spans="1:3">
+      <c r="A29" s="3" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="28" spans="1:3">
-      <c r="A28" t="s">
+      <c r="B29" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B28">
-        <v>1304</v>
-      </c>
-      <c r="C28">
-        <v>1395</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3">
-      <c r="A29" t="s">
+      <c r="C29" s="3" t="s">
         <v>27</v>
-      </c>
-      <c r="B29">
-        <v>1292</v>
-      </c>
-      <c r="C29">
-        <v>1382</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -906,20 +915,42 @@
         <v>28</v>
       </c>
       <c r="B30">
-        <v>312</v>
+        <v>1287</v>
       </c>
       <c r="C30">
-        <v>348</v>
+        <v>1378</v>
       </c>
     </row>
     <row r="31" spans="1:3">
-      <c r="A31" s="5" t="s">
+      <c r="A31" t="s">
         <v>29</v>
       </c>
-      <c r="B31" s="5">
+      <c r="B31">
+        <v>1278</v>
+      </c>
+      <c r="C31">
+        <v>1367</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" t="s">
+        <v>30</v>
+      </c>
+      <c r="B32">
+        <v>343</v>
+      </c>
+      <c r="C32">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B33" s="5">
         <v>2908</v>
       </c>
-      <c r="C31" s="5">
+      <c r="C33" s="5">
         <v>3125</v>
       </c>
     </row>
@@ -938,35 +969,35 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B4" s="4">
         <v>1106</v>
       </c>
       <c r="C4" s="6">
-        <v>0.3803301237964237</v>
+        <v>0.3801652892561984</v>
       </c>
       <c r="D4" s="7">
         <v>414</v>
@@ -977,13 +1008,13 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B5" s="4">
         <v>964</v>
       </c>
       <c r="C5" s="6">
-        <v>0.3314993122420908</v>
+        <v>0.3314967860422406</v>
       </c>
       <c r="D5" s="7">
         <v>361</v>
@@ -994,13 +1025,13 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B6" s="4">
         <v>419</v>
       </c>
       <c r="C6" s="6">
-        <v>0.1440852819807428</v>
+        <v>0.1441689623507805</v>
       </c>
       <c r="D6" s="7">
         <v>157</v>
@@ -1011,13 +1042,13 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B7" s="4">
         <v>243</v>
       </c>
       <c r="C7" s="6">
-        <v>0.08356258596973865</v>
+        <v>0.08356290174471992</v>
       </c>
       <c r="D7" s="7">
         <v>91</v>
@@ -1028,13 +1059,13 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B8" s="4">
         <v>176</v>
       </c>
       <c r="C8" s="6">
-        <v>0.06052269601100413</v>
+        <v>0.06060606060606061</v>
       </c>
       <c r="D8" s="7">
         <v>66</v>
@@ -1045,7 +1076,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B9" s="4">
         <v>2908</v>
@@ -1069,87 +1100,87 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B5" s="8">
         <v>0.15</v>
       </c>
       <c r="C5" s="4">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D5" s="4">
-        <v>204</v>
+        <v>202</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B6" s="8">
         <v>0.33</v>
       </c>
       <c r="C6" s="4">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="D6" s="4">
-        <v>456</v>
+        <v>451</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B7" s="8">
-        <v>0.34</v>
+        <v>0.33</v>
       </c>
       <c r="C7" s="4">
-        <v>437</v>
+        <v>430</v>
       </c>
       <c r="D7" s="4">
-        <v>466</v>
+        <v>458</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B8" s="8">
         <v>0.18</v>
       </c>
       <c r="C8" s="4">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D8" s="4">
-        <v>245</v>
+        <v>242</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B9" s="8">
         <v>0.01</v>
@@ -1163,7 +1194,7 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B10" s="8">
         <v>0</v>
@@ -1172,42 +1203,42 @@
         <v>3</v>
       </c>
       <c r="D10" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B11" s="8">
         <v>1</v>
       </c>
       <c r="C11" s="4">
-        <v>1304</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B15" s="8">
         <v>0.13</v>
@@ -1221,183 +1252,183 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B16" s="8">
         <v>0.25</v>
       </c>
       <c r="C16" s="4">
-        <v>321</v>
+        <v>316</v>
       </c>
       <c r="D16" s="4">
-        <v>343</v>
+        <v>338</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B17" s="8">
         <v>0.3</v>
       </c>
       <c r="C17" s="4">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="D17" s="4">
-        <v>415</v>
+        <v>409</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B18" s="8">
         <v>0.17</v>
       </c>
       <c r="C18" s="4">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="D18" s="4">
-        <v>236</v>
+        <v>234</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B19" s="8">
         <v>0.15</v>
       </c>
       <c r="C19" s="4">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D19" s="4">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B20" s="8">
         <v>1</v>
       </c>
       <c r="C20" s="4">
-        <v>1292</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B24" s="8">
         <v>0.11</v>
       </c>
       <c r="C24" s="4">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="D24" s="4">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B25" s="8">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="C25" s="4">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D25" s="4">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B26" s="8">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
       <c r="C26" s="4">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D26" s="4">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B27" s="8">
         <v>0.21</v>
       </c>
       <c r="C27" s="4">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D27" s="4">
-        <v>73</v>
+        <v>79</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B28" s="8">
         <v>0.22</v>
       </c>
       <c r="C28" s="4">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="D28" s="4">
-        <v>76</v>
+        <v>82</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B29" s="8">
-        <v>0.22</v>
+        <v>0.23</v>
       </c>
       <c r="C29" s="4">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="D29" s="4">
-        <v>76</v>
+        <v>85</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B30" s="8">
         <v>1</v>
       </c>
       <c r="C30" s="4">
-        <v>312</v>
+        <v>343</v>
       </c>
     </row>
   </sheetData>
@@ -1407,107 +1438,170 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C3" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="D3" s="3" t="s">
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B4" s="4">
-        <v>1106</v>
-      </c>
-      <c r="C4" s="7">
-        <v>414</v>
-      </c>
-      <c r="D4" s="7">
-        <v>0.312</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" t="s">
-        <v>37</v>
-      </c>
-      <c r="B5" s="4">
-        <v>964</v>
-      </c>
-      <c r="C5" s="7">
-        <v>361</v>
-      </c>
-      <c r="D5" s="7">
-        <v>0.312</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
+    <row r="5" spans="1:5">
+      <c r="A5" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
       <c r="A6" t="s">
         <v>38</v>
       </c>
       <c r="B6" s="4">
-        <v>419</v>
-      </c>
-      <c r="C6" s="7">
-        <v>157</v>
+        <v>1106</v>
+      </c>
+      <c r="C6" s="6">
+        <v>0.3802</v>
       </c>
       <c r="D6" s="7">
-        <v>0.312</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
+        <v>414</v>
+      </c>
+      <c r="E6" s="7">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
       <c r="A7" t="s">
         <v>39</v>
       </c>
       <c r="B7" s="4">
-        <v>243</v>
-      </c>
-      <c r="C7" s="7">
-        <v>91</v>
+        <v>964</v>
+      </c>
+      <c r="C7" s="6">
+        <v>0.3315</v>
       </c>
       <c r="D7" s="7">
-        <v>0.312</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
+        <v>361</v>
+      </c>
+      <c r="E7" s="7">
+        <v>300.8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
       <c r="A8" t="s">
         <v>40</v>
       </c>
       <c r="B8" s="4">
+        <v>419</v>
+      </c>
+      <c r="C8" s="6">
+        <v>0.1442</v>
+      </c>
+      <c r="D8" s="7">
+        <v>157</v>
+      </c>
+      <c r="E8" s="7">
+        <v>130.8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" s="4">
+        <v>243</v>
+      </c>
+      <c r="C9" s="6">
+        <v>0.08359999999999999</v>
+      </c>
+      <c r="D9" s="7">
+        <v>91</v>
+      </c>
+      <c r="E9" s="7">
+        <v>75.8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="4">
         <v>176</v>
       </c>
-      <c r="C8" s="7">
+      <c r="C10" s="6">
+        <v>0.06059999999999999</v>
+      </c>
+      <c r="D10" s="7">
         <v>66</v>
       </c>
-      <c r="D8" s="7">
-        <v>0.312</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="B9" s="4">
+      <c r="E10" s="7">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B11" s="4">
         <v>2908</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C11" s="8">
+        <v>1</v>
+      </c>
+      <c r="D11" s="7">
         <v>1089</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17">
+        <v>0.22</v>
       </c>
     </row>
   </sheetData>
@@ -1522,72 +1616,72 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="2" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="3" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B5" s="7">
         <v>361.2</v>
       </c>
       <c r="C5" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="B6" s="7">
         <v>125.1</v>
       </c>
       <c r="C6" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="B7" s="7">
         <v>157</v>
       </c>
       <c r="C7" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="B8" s="7">
         <v>62.8</v>
       </c>
       <c r="C8" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="5" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="B9" s="7">
         <v>706.1</v>
@@ -1595,67 +1689,67 @@
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="2" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="3" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="B13" s="7">
         <v>157</v>
       </c>
       <c r="C13" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B14" s="7">
         <v>94.2</v>
       </c>
       <c r="C14" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="B15" s="7">
         <v>65.59999999999999</v>
       </c>
       <c r="C15" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B16" s="7">
         <v>65.5</v>
       </c>
       <c r="C16" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="5" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="B17" s="7">
         <v>382.3</v>
@@ -1663,7 +1757,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="5" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="B19" s="7">
         <v>1088.4</v>
@@ -1681,78 +1775,78 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="3" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B5">
         <v>63</v>
       </c>
       <c r="C5">
+        <v>158</v>
+      </c>
+      <c r="D5">
         <v>159</v>
       </c>
-      <c r="D5">
-        <v>161</v>
-      </c>
       <c r="E5">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F5">
         <v>12</v>
       </c>
       <c r="G5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H5">
-        <v>484</v>
+        <v>479</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B6">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C6">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D6">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="E6">
         <v>71</v>
@@ -1764,12 +1858,12 @@
         <v>0</v>
       </c>
       <c r="H6">
-        <v>441</v>
+        <v>436</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B7">
         <v>31</v>
@@ -1778,10 +1872,10 @@
         <v>65</v>
       </c>
       <c r="D7">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E7">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F7">
         <v>3</v>
@@ -1790,21 +1884,21 @@
         <v>0</v>
       </c>
       <c r="H7">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B8">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C8">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D8">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E8">
         <v>19</v>
@@ -1816,112 +1910,112 @@
         <v>0</v>
       </c>
       <c r="H8">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B9">
         <v>9</v>
       </c>
       <c r="C9">
+        <v>26</v>
+      </c>
+      <c r="D9">
         <v>27</v>
       </c>
-      <c r="D9">
-        <v>28</v>
-      </c>
       <c r="E9">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F9">
         <v>0</v>
       </c>
       <c r="G9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H9">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" s="3" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B13">
         <v>80</v>
       </c>
       <c r="C13">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D13">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="E13">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F13">
         <v>75</v>
       </c>
       <c r="G13">
-        <v>510</v>
+        <v>505</v>
       </c>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B14">
         <v>51</v>
       </c>
       <c r="C14">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D14">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E14">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F14">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G14">
-        <v>428</v>
+        <v>423</v>
       </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B15">
         <v>22</v>
@@ -1930,7 +2024,7 @@
         <v>52</v>
       </c>
       <c r="D15">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E15">
         <v>38</v>
@@ -1939,18 +2033,18 @@
         <v>26</v>
       </c>
       <c r="G15">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B16">
         <v>7</v>
       </c>
       <c r="C16">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D16">
         <v>31</v>
@@ -1959,21 +2053,21 @@
         <v>16</v>
       </c>
       <c r="F16">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G16">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B17">
         <v>7</v>
       </c>
       <c r="C17">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D17">
         <v>18</v>
@@ -1985,130 +2079,130 @@
         <v>9</v>
       </c>
       <c r="G17">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:8">
       <c r="A20" s="3" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
     </row>
     <row r="21" spans="1:8">
       <c r="A21" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B21">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C21">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D21">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E21">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F21">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G21">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="H21">
-        <v>111</v>
+        <v>122</v>
       </c>
     </row>
     <row r="22" spans="1:8">
       <c r="A22" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B22">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C22">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D22">
         <v>8</v>
       </c>
       <c r="E22">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F22">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G22">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H22">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="23" spans="1:8">
       <c r="A23" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B23">
         <v>4</v>
       </c>
       <c r="C23">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D23">
         <v>5</v>
       </c>
       <c r="E23">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F23">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G23">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H23">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="24" spans="1:8">
       <c r="A24" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B24">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C24">
         <v>4</v>
       </c>
       <c r="D24">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E24">
         <v>7</v>
@@ -2117,21 +2211,21 @@
         <v>7</v>
       </c>
       <c r="G24">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H24">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="25" spans="1:8">
       <c r="A25" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B25">
         <v>2</v>
       </c>
       <c r="C25">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D25">
         <v>3</v>
@@ -2143,10 +2237,10 @@
         <v>5</v>
       </c>
       <c r="G25">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H25">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -2156,7 +2250,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="100.7109375" customWidth="1"/>
@@ -2164,32 +2258,42 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>97</v>
+        <v>102</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9" t="s">
+        <v>104</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Explore Pants: CAB sin 3XL, más KIDS y boost Kaki/Azul/Verde
- Excluye 3XL en caballero
- KIDS gender boost 1.12 → 1.18 (+26 und aprox.)
- Color boost: Kaki +10%, Azul Marino +15%, Verde Militar +15%

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/EXPLORE_PANTS_Proyeccion_Produccion.xlsx
+++ b/EXPLORE_PANTS_Proyeccion_Produccion.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="104">
   <si>
     <t>EXPLORE PANTS — PROYECCIÓN ANCLADA A JUSTIFICACIÓN NOVAKTEX</t>
   </si>
@@ -46,10 +46,10 @@
     <t>Pedido total archivo (Explore + Shorts): 1088 kg · split 65% / 35%</t>
   </si>
   <si>
-    <t>Color: proporción del pedido (Negro 38% · Gris Oscuro 33% · Kaki 14% · Azul 8% · Verde 6%)</t>
-  </si>
-  <si>
-    <t>Talla/género: curva de ventas del dashboard · KIDS con boost moderado (+12%)</t>
+    <t>Color: base compra + boost Kaki/Azul/Verde para no dejarlos tan bajos</t>
+  </si>
+  <si>
+    <t>Talla/género: curva ventas · KIDS +17% · CAB sin 3XL</t>
   </si>
   <si>
     <t>Consumo referencial: CAB 0.3 · DAMA 0.25 · KIDS 0.22 kg/und</t>
@@ -127,7 +127,7 @@
     <t>Und a producir</t>
   </si>
   <si>
-    <t>% compra (color)</t>
+    <t>% producción</t>
   </si>
   <si>
     <t>Kg tela comprada (ref.)</t>
@@ -184,9 +184,6 @@
     <t>2XL</t>
   </si>
   <si>
-    <t>3XL</t>
-  </si>
-  <si>
     <t>DAMA — TALLAS</t>
   </si>
   <si>
@@ -319,16 +316,16 @@
     <t>1. TOTAL a producir: 2,908 und (80% pendiente, justificación Novaktex). La tela ya está comprada.</t>
   </si>
   <si>
-    <t>2. COLOR: proporción del pedido de tela — Negro 38.0% · Gris Oscuro 33.1% · Kaki 14.4% · Azul Marino 8.4% · Verde Militar 6.1%.</t>
-  </si>
-  <si>
-    <t>3. GÉNERO y TALLA: curva de ventas del dashboard dentro de cada color; KIDS con boost +12% sobre su share de ventas.</t>
+    <t>2. COLOR: base compra + boost Kaki +10% · Azul Marino +15% · Verde Militar +15% → Negro 36.7% · Gris Oscuro 32.0% · Kaki 15.3% · Azul Marino 9.3% · Verde Militar 6.7%.</t>
+  </si>
+  <si>
+    <t>3. GÉNERO y TALLA: curva ventas por color; KIDS +17%; CAB sin 3XL; KIDS sin talla 1.</t>
   </si>
   <si>
     <t>4. Consumo referencial (no define und): CAB 0.3 · DAMA 0.25 · KIDS 0.22 kg/und.</t>
   </si>
   <si>
-    <t>5. KIDS excluye talla 1 en producción (venta marginal). Gris (ventas) → Gris Oscuro (producción).</t>
+    <t>5. Gris (ventas) → Gris Oscuro (producción).</t>
   </si>
   <si>
     <t>6. Demanda Jul–Dic (2,228 und) y escenarios mensuales del archivo de justificación.</t>
@@ -915,10 +912,10 @@
         <v>28</v>
       </c>
       <c r="B30">
-        <v>1287</v>
+        <v>1279</v>
       </c>
       <c r="C30">
-        <v>1378</v>
+        <v>1367</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -926,10 +923,10 @@
         <v>29</v>
       </c>
       <c r="B31">
-        <v>1278</v>
+        <v>1264</v>
       </c>
       <c r="C31">
-        <v>1367</v>
+        <v>1354</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -937,10 +934,10 @@
         <v>30</v>
       </c>
       <c r="B32">
-        <v>343</v>
+        <v>365</v>
       </c>
       <c r="C32">
-        <v>380</v>
+        <v>403</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -951,7 +948,7 @@
         <v>2908</v>
       </c>
       <c r="C33" s="5">
-        <v>3125</v>
+        <v>3124</v>
       </c>
     </row>
   </sheetData>
@@ -994,10 +991,10 @@
         <v>38</v>
       </c>
       <c r="B4" s="4">
-        <v>1106</v>
+        <v>1067</v>
       </c>
       <c r="C4" s="6">
-        <v>0.3801652892561984</v>
+        <v>0.3669399512519388</v>
       </c>
       <c r="D4" s="7">
         <v>414</v>
@@ -1011,10 +1008,10 @@
         <v>39</v>
       </c>
       <c r="B5" s="4">
-        <v>964</v>
+        <v>930</v>
       </c>
       <c r="C5" s="6">
-        <v>0.3314967860422406</v>
+        <v>0.3199645468646133</v>
       </c>
       <c r="D5" s="7">
         <v>361</v>
@@ -1028,10 +1025,10 @@
         <v>40</v>
       </c>
       <c r="B6" s="4">
-        <v>419</v>
+        <v>445</v>
       </c>
       <c r="C6" s="6">
-        <v>0.1441689623507805</v>
+        <v>0.1530689120319078</v>
       </c>
       <c r="D6" s="7">
         <v>157</v>
@@ -1045,10 +1042,10 @@
         <v>41</v>
       </c>
       <c r="B7" s="4">
-        <v>243</v>
+        <v>270</v>
       </c>
       <c r="C7" s="6">
-        <v>0.08356290174471992</v>
+        <v>0.09275426545535119</v>
       </c>
       <c r="D7" s="7">
         <v>91</v>
@@ -1062,10 +1059,10 @@
         <v>42</v>
       </c>
       <c r="B8" s="4">
-        <v>176</v>
+        <v>196</v>
       </c>
       <c r="C8" s="6">
-        <v>0.06060606060606061</v>
+        <v>0.06727232439618877</v>
       </c>
       <c r="D8" s="7">
         <v>66</v>
@@ -1095,7 +1092,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -1130,10 +1127,10 @@
         <v>0.15</v>
       </c>
       <c r="C5" s="4">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D5" s="4">
-        <v>202</v>
+        <v>200</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -1144,10 +1141,10 @@
         <v>0.33</v>
       </c>
       <c r="C6" s="4">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D6" s="4">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -1155,7 +1152,7 @@
         <v>51</v>
       </c>
       <c r="B7" s="8">
-        <v>0.33</v>
+        <v>0.34</v>
       </c>
       <c r="C7" s="4">
         <v>430</v>
@@ -1172,10 +1169,10 @@
         <v>0.18</v>
       </c>
       <c r="C8" s="4">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D8" s="4">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -1186,154 +1183,154 @@
         <v>0.01</v>
       </c>
       <c r="C9" s="4">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D9" s="4">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:4">
-      <c r="A10" t="s">
+      <c r="A10" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="8">
+        <v>1</v>
+      </c>
+      <c r="C10" s="4">
+        <v>1279</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B10" s="8">
-        <v>0</v>
-      </c>
-      <c r="C10" s="4">
-        <v>3</v>
-      </c>
-      <c r="D10" s="4">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B11" s="8">
-        <v>1</v>
-      </c>
-      <c r="C11" s="4">
-        <v>1287</v>
-      </c>
     </row>
     <row r="13" spans="1:4">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>48</v>
+      <c r="B14" s="8">
+        <v>0.13</v>
+      </c>
+      <c r="C14" s="4">
+        <v>163</v>
+      </c>
+      <c r="D14" s="4">
+        <v>175</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="B15" s="8">
-        <v>0.13</v>
+        <v>0.25</v>
       </c>
       <c r="C15" s="4">
-        <v>167</v>
+        <v>312</v>
       </c>
       <c r="D15" s="4">
-        <v>180</v>
+        <v>335</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B16" s="8">
-        <v>0.25</v>
+        <v>0.3</v>
       </c>
       <c r="C16" s="4">
-        <v>316</v>
+        <v>381</v>
       </c>
       <c r="D16" s="4">
-        <v>338</v>
+        <v>406</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B17" s="8">
-        <v>0.3</v>
+        <v>0.17</v>
       </c>
       <c r="C17" s="4">
-        <v>384</v>
+        <v>217</v>
       </c>
       <c r="D17" s="4">
-        <v>409</v>
+        <v>233</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B18" s="8">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
       <c r="C18" s="4">
-        <v>219</v>
+        <v>191</v>
       </c>
       <c r="D18" s="4">
-        <v>234</v>
+        <v>205</v>
       </c>
     </row>
     <row r="19" spans="1:4">
-      <c r="A19" t="s">
-        <v>52</v>
+      <c r="A19" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="B19" s="8">
-        <v>0.15</v>
+        <v>1</v>
       </c>
       <c r="C19" s="4">
-        <v>192</v>
-      </c>
-      <c r="D19" s="4">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4">
-      <c r="A20" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B20" s="8">
-        <v>1</v>
-      </c>
-      <c r="C20" s="4">
-        <v>1278</v>
+        <v>1264</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" s="2" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="22" spans="1:4">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="23" spans="1:4">
-      <c r="A23" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>48</v>
+      <c r="B23" s="8">
+        <v>0.1</v>
+      </c>
+      <c r="C23" s="4">
+        <v>38</v>
+      </c>
+      <c r="D23" s="4">
+        <v>44</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -1341,13 +1338,13 @@
         <v>58</v>
       </c>
       <c r="B24" s="8">
-        <v>0.11</v>
+        <v>0.13</v>
       </c>
       <c r="C24" s="4">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="D24" s="4">
-        <v>43</v>
+        <v>53</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -1355,13 +1352,13 @@
         <v>59</v>
       </c>
       <c r="B25" s="8">
-        <v>0.13</v>
+        <v>0.11</v>
       </c>
       <c r="C25" s="4">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="D25" s="4">
-        <v>51</v>
+        <v>44</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -1369,13 +1366,13 @@
         <v>60</v>
       </c>
       <c r="B26" s="8">
-        <v>0.1</v>
+        <v>0.21</v>
       </c>
       <c r="C26" s="4">
-        <v>35</v>
+        <v>76</v>
       </c>
       <c r="D26" s="4">
-        <v>40</v>
+        <v>83</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -1383,13 +1380,13 @@
         <v>61</v>
       </c>
       <c r="B27" s="8">
-        <v>0.21</v>
+        <v>0.22</v>
       </c>
       <c r="C27" s="4">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="D27" s="4">
-        <v>79</v>
+        <v>88</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -1397,38 +1394,24 @@
         <v>62</v>
       </c>
       <c r="B28" s="8">
-        <v>0.22</v>
+        <v>0.23</v>
       </c>
       <c r="C28" s="4">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="D28" s="4">
-        <v>82</v>
+        <v>91</v>
       </c>
     </row>
     <row r="29" spans="1:4">
-      <c r="A29" t="s">
-        <v>63</v>
+      <c r="A29" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="B29" s="8">
-        <v>0.23</v>
+        <v>1</v>
       </c>
       <c r="C29" s="4">
-        <v>78</v>
-      </c>
-      <c r="D29" s="4">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4">
-      <c r="A30" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B30" s="8">
-        <v>1</v>
-      </c>
-      <c r="C30" s="4">
-        <v>343</v>
+        <v>365</v>
       </c>
     </row>
   </sheetData>
@@ -1443,12 +1426,12 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -1459,13 +1442,13 @@
         <v>34</v>
       </c>
       <c r="C5" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>67</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -1473,10 +1456,10 @@
         <v>38</v>
       </c>
       <c r="B6" s="4">
-        <v>1106</v>
+        <v>1067</v>
       </c>
       <c r="C6" s="6">
-        <v>0.3802</v>
+        <v>0.3669</v>
       </c>
       <c r="D6" s="7">
         <v>414</v>
@@ -1490,10 +1473,10 @@
         <v>39</v>
       </c>
       <c r="B7" s="4">
-        <v>964</v>
+        <v>930</v>
       </c>
       <c r="C7" s="6">
-        <v>0.3315</v>
+        <v>0.32</v>
       </c>
       <c r="D7" s="7">
         <v>361</v>
@@ -1507,10 +1490,10 @@
         <v>40</v>
       </c>
       <c r="B8" s="4">
-        <v>419</v>
+        <v>445</v>
       </c>
       <c r="C8" s="6">
-        <v>0.1442</v>
+        <v>0.1531</v>
       </c>
       <c r="D8" s="7">
         <v>157</v>
@@ -1524,10 +1507,10 @@
         <v>41</v>
       </c>
       <c r="B9" s="4">
-        <v>243</v>
+        <v>270</v>
       </c>
       <c r="C9" s="6">
-        <v>0.08359999999999999</v>
+        <v>0.09279999999999999</v>
       </c>
       <c r="D9" s="7">
         <v>91</v>
@@ -1541,10 +1524,10 @@
         <v>42</v>
       </c>
       <c r="B10" s="4">
-        <v>176</v>
+        <v>196</v>
       </c>
       <c r="C10" s="6">
-        <v>0.06059999999999999</v>
+        <v>0.0673</v>
       </c>
       <c r="D10" s="7">
         <v>66</v>
@@ -1555,7 +1538,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B11" s="4">
         <v>2908</v>
@@ -1569,7 +1552,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -1577,7 +1560,7 @@
         <v>25</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -1616,72 +1599,72 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>75</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B5" s="7">
         <v>361.2</v>
       </c>
       <c r="C5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B6" s="7">
         <v>125.1</v>
       </c>
       <c r="C6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B7" s="7">
         <v>157</v>
       </c>
       <c r="C7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B8" s="7">
         <v>62.8</v>
       </c>
       <c r="C8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B9" s="7">
         <v>706.1</v>
@@ -1689,67 +1672,67 @@
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>75</v>
-      </c>
       <c r="C12" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B13" s="7">
         <v>157</v>
       </c>
       <c r="C13" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B14" s="7">
         <v>94.2</v>
       </c>
       <c r="C14" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B15" s="7">
         <v>65.59999999999999</v>
       </c>
       <c r="C15" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B16" s="7">
         <v>65.5</v>
       </c>
       <c r="C16" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B17" s="7">
         <v>382.3</v>
@@ -1757,7 +1740,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B19" s="7">
         <v>1088.4</v>
@@ -1773,19 +1756,19 @@
   <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
       <c r="A3" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:7">
       <c r="A4" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>49</v>
@@ -1803,153 +1786,135 @@
         <v>53</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
       <c r="A5" t="s">
         <v>38</v>
       </c>
       <c r="B5">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C5">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="D5">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="E5">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="F5">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G5">
-        <v>2</v>
-      </c>
-      <c r="H5">
-        <v>479</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
       <c r="A6" t="s">
         <v>39</v>
       </c>
       <c r="B6">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C6">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="D6">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="E6">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F6">
         <v>2</v>
       </c>
       <c r="G6">
-        <v>0</v>
-      </c>
-      <c r="H6">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
       <c r="A7" t="s">
         <v>40</v>
       </c>
       <c r="B7">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C7">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D7">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="E7">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F7">
         <v>3</v>
       </c>
       <c r="G7">
-        <v>0</v>
-      </c>
-      <c r="H7">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>41</v>
       </c>
       <c r="B8">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C8">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="D8">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E8">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F8">
         <v>0</v>
       </c>
       <c r="G8">
-        <v>0</v>
-      </c>
-      <c r="H8">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
       <c r="A9" t="s">
         <v>42</v>
       </c>
       <c r="B9">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C9">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D9">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E9">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F9">
         <v>0</v>
       </c>
       <c r="G9">
-        <v>1</v>
-      </c>
-      <c r="H9">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
       <c r="A11" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:7">
       <c r="A12" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>49</v>
@@ -1964,99 +1929,99 @@
         <v>52</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
       <c r="A13" t="s">
         <v>38</v>
       </c>
       <c r="B13">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C13">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="D13">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="E13">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="F13">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="G13">
-        <v>505</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
       <c r="A14" t="s">
         <v>39</v>
       </c>
       <c r="B14">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C14">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="D14">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="E14">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="F14">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="G14">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
       <c r="A15" t="s">
         <v>40</v>
       </c>
       <c r="B15">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C15">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D15">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E15">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F15">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G15">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
       <c r="A16" t="s">
         <v>41</v>
       </c>
       <c r="B16">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C16">
+        <v>19</v>
+      </c>
+      <c r="D16">
+        <v>33</v>
+      </c>
+      <c r="E16">
         <v>17</v>
       </c>
-      <c r="D16">
-        <v>31</v>
-      </c>
-      <c r="E16">
-        <v>16</v>
-      </c>
       <c r="F16">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G16">
-        <v>88</v>
+        <v>96</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -2067,19 +2032,19 @@
         <v>7</v>
       </c>
       <c r="C17">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D17">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E17">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F17">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G17">
-        <v>62</v>
+        <v>68</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -2089,28 +2054,28 @@
     </row>
     <row r="20" spans="1:8">
       <c r="A20" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="H20" s="3" t="s">
         <v>95</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="H20" s="3" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -2124,19 +2089,19 @@
         <v>16</v>
       </c>
       <c r="D21">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E21">
         <v>23</v>
       </c>
       <c r="F21">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G21">
         <v>25</v>
       </c>
       <c r="H21">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -2150,7 +2115,7 @@
         <v>13</v>
       </c>
       <c r="D22">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E22">
         <v>29</v>
@@ -2159,10 +2124,10 @@
         <v>23</v>
       </c>
       <c r="G22">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H22">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -2170,25 +2135,25 @@
         <v>41</v>
       </c>
       <c r="B23">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C23">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D23">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E23">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F23">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G23">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H23">
-        <v>55</v>
+        <v>64</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -2199,22 +2164,22 @@
         <v>3</v>
       </c>
       <c r="C24">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D24">
         <v>6</v>
       </c>
       <c r="E24">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F24">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G24">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H24">
-        <v>37</v>
+        <v>43</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -2228,19 +2193,19 @@
         <v>5</v>
       </c>
       <c r="D25">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E25">
         <v>3</v>
       </c>
       <c r="F25">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G25">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H25">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -2258,42 +2223,42 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Explore Pants: KIDS meta 500 und
- Meta explícita KIDS=500; CAB/DAMA reparten el resto por ventas
- Corrige referencias rotas a KIDS_GENDER_BOOST en dashboard/Excel

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/EXPLORE_PANTS_Proyeccion_Produccion.xlsx
+++ b/EXPLORE_PANTS_Proyeccion_Produccion.xlsx
@@ -49,7 +49,7 @@
     <t>Color: base compra + boost Kaki/Azul/Verde para no dejarlos tan bajos</t>
   </si>
   <si>
-    <t>Talla/género: curva ventas · KIDS +17% · CAB sin 3XL</t>
+    <t>Talla/género: curva ventas · KIDS meta 500 und · CAB sin 3XL</t>
   </si>
   <si>
     <t>Consumo referencial: CAB 0.3 · DAMA 0.25 · KIDS 0.22 kg/und</t>
@@ -319,7 +319,7 @@
     <t>2. COLOR: base compra + boost Kaki +10% · Azul Marino +15% · Verde Militar +15% → Negro 36.7% · Gris Oscuro 32.0% · Kaki 15.3% · Azul Marino 9.3% · Verde Militar 6.7%.</t>
   </si>
   <si>
-    <t>3. GÉNERO y TALLA: curva ventas por color; KIDS +17%; CAB sin 3XL; KIDS sin talla 1.</t>
+    <t>3. GÉNERO y TALLA: curva ventas por color; KIDS meta 500 und; CAB sin 3XL; KIDS sin talla 1.</t>
   </si>
   <si>
     <t>4. Consumo referencial (no define und): CAB 0.3 · DAMA 0.25 · KIDS 0.22 kg/und.</t>
@@ -912,10 +912,10 @@
         <v>28</v>
       </c>
       <c r="B30">
-        <v>1279</v>
+        <v>1209</v>
       </c>
       <c r="C30">
-        <v>1367</v>
+        <v>1293</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -923,10 +923,10 @@
         <v>29</v>
       </c>
       <c r="B31">
-        <v>1264</v>
+        <v>1199</v>
       </c>
       <c r="C31">
-        <v>1354</v>
+        <v>1283</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -934,10 +934,10 @@
         <v>30</v>
       </c>
       <c r="B32">
-        <v>365</v>
+        <v>500</v>
       </c>
       <c r="C32">
-        <v>403</v>
+        <v>545</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -948,7 +948,7 @@
         <v>2908</v>
       </c>
       <c r="C33" s="5">
-        <v>3124</v>
+        <v>3121</v>
       </c>
     </row>
   </sheetData>
@@ -1127,10 +1127,10 @@
         <v>0.15</v>
       </c>
       <c r="C5" s="4">
-        <v>187</v>
+        <v>177</v>
       </c>
       <c r="D5" s="4">
-        <v>200</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -1141,10 +1141,10 @@
         <v>0.33</v>
       </c>
       <c r="C6" s="4">
-        <v>422</v>
+        <v>398</v>
       </c>
       <c r="D6" s="4">
-        <v>450</v>
+        <v>425</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -1155,10 +1155,10 @@
         <v>0.34</v>
       </c>
       <c r="C7" s="4">
-        <v>430</v>
+        <v>406</v>
       </c>
       <c r="D7" s="4">
-        <v>458</v>
+        <v>432</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -1169,10 +1169,10 @@
         <v>0.18</v>
       </c>
       <c r="C8" s="4">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="D8" s="4">
-        <v>240</v>
+        <v>227</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -1197,7 +1197,7 @@
         <v>1</v>
       </c>
       <c r="C10" s="4">
-        <v>1279</v>
+        <v>1209</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -1227,10 +1227,10 @@
         <v>0.13</v>
       </c>
       <c r="C14" s="4">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="D14" s="4">
-        <v>175</v>
+        <v>167</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -1241,10 +1241,10 @@
         <v>0.25</v>
       </c>
       <c r="C15" s="4">
-        <v>312</v>
+        <v>297</v>
       </c>
       <c r="D15" s="4">
-        <v>335</v>
+        <v>317</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -1255,10 +1255,10 @@
         <v>0.3</v>
       </c>
       <c r="C16" s="4">
-        <v>381</v>
+        <v>361</v>
       </c>
       <c r="D16" s="4">
-        <v>406</v>
+        <v>385</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -1269,10 +1269,10 @@
         <v>0.17</v>
       </c>
       <c r="C17" s="4">
-        <v>217</v>
+        <v>206</v>
       </c>
       <c r="D17" s="4">
-        <v>233</v>
+        <v>221</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -1283,10 +1283,10 @@
         <v>0.15</v>
       </c>
       <c r="C18" s="4">
-        <v>191</v>
+        <v>180</v>
       </c>
       <c r="D18" s="4">
-        <v>205</v>
+        <v>193</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -1297,7 +1297,7 @@
         <v>1</v>
       </c>
       <c r="C19" s="4">
-        <v>1264</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -1324,13 +1324,13 @@
         <v>57</v>
       </c>
       <c r="B23" s="8">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="C23" s="4">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="D23" s="4">
-        <v>44</v>
+        <v>59</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -1341,10 +1341,10 @@
         <v>0.13</v>
       </c>
       <c r="C24" s="4">
-        <v>48</v>
+        <v>66</v>
       </c>
       <c r="D24" s="4">
-        <v>53</v>
+        <v>73</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -1355,10 +1355,10 @@
         <v>0.11</v>
       </c>
       <c r="C25" s="4">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="D25" s="4">
-        <v>44</v>
+        <v>59</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -1369,10 +1369,10 @@
         <v>0.21</v>
       </c>
       <c r="C26" s="4">
-        <v>76</v>
+        <v>105</v>
       </c>
       <c r="D26" s="4">
-        <v>83</v>
+        <v>113</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -1383,10 +1383,10 @@
         <v>0.22</v>
       </c>
       <c r="C27" s="4">
-        <v>81</v>
+        <v>108</v>
       </c>
       <c r="D27" s="4">
-        <v>88</v>
+        <v>117</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -1397,10 +1397,10 @@
         <v>0.23</v>
       </c>
       <c r="C28" s="4">
-        <v>83</v>
+        <v>115</v>
       </c>
       <c r="D28" s="4">
-        <v>91</v>
+        <v>124</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -1411,7 +1411,7 @@
         <v>1</v>
       </c>
       <c r="C29" s="4">
-        <v>365</v>
+        <v>500</v>
       </c>
     </row>
   </sheetData>
@@ -1794,22 +1794,22 @@
         <v>38</v>
       </c>
       <c r="B5">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C5">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="D5">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="E5">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="F5">
         <v>11</v>
       </c>
       <c r="G5">
-        <v>459</v>
+        <v>437</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -1817,22 +1817,22 @@
         <v>39</v>
       </c>
       <c r="B6">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C6">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="D6">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="E6">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F6">
         <v>2</v>
       </c>
       <c r="G6">
-        <v>418</v>
+        <v>398</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -1840,22 +1840,22 @@
         <v>40</v>
       </c>
       <c r="B7">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C7">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D7">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E7">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F7">
         <v>3</v>
       </c>
       <c r="G7">
-        <v>207</v>
+        <v>202</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -1863,22 +1863,22 @@
         <v>41</v>
       </c>
       <c r="B8">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C8">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="D8">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="E8">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F8">
         <v>0</v>
       </c>
       <c r="G8">
-        <v>110</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -1886,22 +1886,22 @@
         <v>42</v>
       </c>
       <c r="B9">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C9">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D9">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E9">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F9">
         <v>0</v>
       </c>
       <c r="G9">
-        <v>85</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -1937,22 +1937,22 @@
         <v>38</v>
       </c>
       <c r="B13">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C13">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="D13">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="E13">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="F13">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="G13">
-        <v>484</v>
+        <v>461</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -1960,22 +1960,22 @@
         <v>39</v>
       </c>
       <c r="B14">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C14">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="D14">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="E14">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="F14">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="G14">
-        <v>405</v>
+        <v>386</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -1983,22 +1983,22 @@
         <v>40</v>
       </c>
       <c r="B15">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C15">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D15">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E15">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F15">
         <v>27</v>
       </c>
       <c r="G15">
-        <v>211</v>
+        <v>207</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -2006,22 +2006,22 @@
         <v>41</v>
       </c>
       <c r="B16">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C16">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D16">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E16">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F16">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G16">
-        <v>96</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -2029,22 +2029,22 @@
         <v>42</v>
       </c>
       <c r="B17">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C17">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D17">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E17">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F17">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G17">
-        <v>68</v>
+        <v>61</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -2083,25 +2083,25 @@
         <v>38</v>
       </c>
       <c r="B21">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C21">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D21">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="E21">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="F21">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="G21">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="H21">
-        <v>124</v>
+        <v>169</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -2109,25 +2109,25 @@
         <v>39</v>
       </c>
       <c r="B22">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C22">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="D22">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E22">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="F22">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="G22">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="H22">
-        <v>107</v>
+        <v>146</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -2135,25 +2135,25 @@
         <v>41</v>
       </c>
       <c r="B23">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C23">
+        <v>12</v>
+      </c>
+      <c r="D23">
         <v>9</v>
       </c>
-      <c r="D23">
-        <v>6</v>
-      </c>
       <c r="E23">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F23">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="G23">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="H23">
-        <v>64</v>
+        <v>89</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -2161,25 +2161,25 @@
         <v>42</v>
       </c>
       <c r="B24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C24">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D24">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E24">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F24">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G24">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="H24">
-        <v>43</v>
+        <v>60</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -2187,25 +2187,25 @@
         <v>40</v>
       </c>
       <c r="B25">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C25">
+        <v>7</v>
+      </c>
+      <c r="D25">
         <v>5</v>
       </c>
-      <c r="D25">
-        <v>4</v>
-      </c>
       <c r="E25">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F25">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G25">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H25">
-        <v>27</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Explore Pants: KIDS 550–620 und (meta 585)
Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/EXPLORE_PANTS_Proyeccion_Produccion.xlsx
+++ b/EXPLORE_PANTS_Proyeccion_Produccion.xlsx
@@ -49,7 +49,7 @@
     <t>Color: base compra + boost Kaki/Azul/Verde para no dejarlos tan bajos</t>
   </si>
   <si>
-    <t>Talla/género: curva ventas · KIDS meta 500 und · CAB sin 3XL</t>
+    <t>Talla/género: curva ventas · KIDS 550–620 und · CAB sin 3XL</t>
   </si>
   <si>
     <t>Consumo referencial: CAB 0.3 · DAMA 0.25 · KIDS 0.22 kg/und</t>
@@ -319,7 +319,7 @@
     <t>2. COLOR: base compra + boost Kaki +10% · Azul Marino +15% · Verde Militar +15% → Negro 36.7% · Gris Oscuro 32.0% · Kaki 15.3% · Azul Marino 9.3% · Verde Militar 6.7%.</t>
   </si>
   <si>
-    <t>3. GÉNERO y TALLA: curva ventas por color; KIDS meta 500 und; CAB sin 3XL; KIDS sin talla 1.</t>
+    <t>3. GÉNERO y TALLA: curva ventas por color; KIDS 550–620 und (meta 585); CAB sin 3XL; KIDS sin talla 1.</t>
   </si>
   <si>
     <t>4. Consumo referencial (no define und): CAB 0.3 · DAMA 0.25 · KIDS 0.22 kg/und.</t>
@@ -912,10 +912,10 @@
         <v>28</v>
       </c>
       <c r="B30">
-        <v>1209</v>
+        <v>1166</v>
       </c>
       <c r="C30">
-        <v>1293</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -923,10 +923,10 @@
         <v>29</v>
       </c>
       <c r="B31">
-        <v>1199</v>
+        <v>1157</v>
       </c>
       <c r="C31">
-        <v>1283</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -934,10 +934,10 @@
         <v>30</v>
       </c>
       <c r="B32">
-        <v>500</v>
+        <v>585</v>
       </c>
       <c r="C32">
-        <v>545</v>
+        <v>636</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -948,7 +948,7 @@
         <v>2908</v>
       </c>
       <c r="C33" s="5">
-        <v>3121</v>
+        <v>3118</v>
       </c>
     </row>
   </sheetData>
@@ -1127,10 +1127,10 @@
         <v>0.15</v>
       </c>
       <c r="C5" s="4">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="D5" s="4">
-        <v>190</v>
+        <v>183</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -1141,10 +1141,10 @@
         <v>0.33</v>
       </c>
       <c r="C6" s="4">
-        <v>398</v>
+        <v>384</v>
       </c>
       <c r="D6" s="4">
-        <v>425</v>
+        <v>409</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -1155,10 +1155,10 @@
         <v>0.34</v>
       </c>
       <c r="C7" s="4">
-        <v>406</v>
+        <v>392</v>
       </c>
       <c r="D7" s="4">
-        <v>432</v>
+        <v>417</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -1166,13 +1166,13 @@
         <v>52</v>
       </c>
       <c r="B8" s="8">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="C8" s="4">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="D8" s="4">
-        <v>227</v>
+        <v>217</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -1197,7 +1197,7 @@
         <v>1</v>
       </c>
       <c r="C10" s="4">
-        <v>1209</v>
+        <v>1166</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -1227,10 +1227,10 @@
         <v>0.13</v>
       </c>
       <c r="C14" s="4">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="D14" s="4">
-        <v>167</v>
+        <v>161</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -1241,10 +1241,10 @@
         <v>0.25</v>
       </c>
       <c r="C15" s="4">
-        <v>297</v>
+        <v>288</v>
       </c>
       <c r="D15" s="4">
-        <v>317</v>
+        <v>307</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -1255,10 +1255,10 @@
         <v>0.3</v>
       </c>
       <c r="C16" s="4">
-        <v>361</v>
+        <v>348</v>
       </c>
       <c r="D16" s="4">
-        <v>385</v>
+        <v>370</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -1269,10 +1269,10 @@
         <v>0.17</v>
       </c>
       <c r="C17" s="4">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="D17" s="4">
-        <v>221</v>
+        <v>214</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -1283,10 +1283,10 @@
         <v>0.15</v>
       </c>
       <c r="C18" s="4">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="D18" s="4">
-        <v>193</v>
+        <v>185</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -1297,7 +1297,7 @@
         <v>1</v>
       </c>
       <c r="C19" s="4">
-        <v>1199</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -1327,10 +1327,10 @@
         <v>0.11</v>
       </c>
       <c r="C23" s="4">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="D23" s="4">
-        <v>59</v>
+        <v>69</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -1341,10 +1341,10 @@
         <v>0.13</v>
       </c>
       <c r="C24" s="4">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="D24" s="4">
-        <v>73</v>
+        <v>84</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -1352,13 +1352,13 @@
         <v>59</v>
       </c>
       <c r="B25" s="8">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
       <c r="C25" s="4">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="D25" s="4">
-        <v>59</v>
+        <v>67</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -1369,10 +1369,10 @@
         <v>0.21</v>
       </c>
       <c r="C26" s="4">
-        <v>105</v>
+        <v>122</v>
       </c>
       <c r="D26" s="4">
-        <v>113</v>
+        <v>132</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -1383,10 +1383,10 @@
         <v>0.22</v>
       </c>
       <c r="C27" s="4">
-        <v>108</v>
+        <v>129</v>
       </c>
       <c r="D27" s="4">
-        <v>117</v>
+        <v>139</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -1397,10 +1397,10 @@
         <v>0.23</v>
       </c>
       <c r="C28" s="4">
-        <v>115</v>
+        <v>134</v>
       </c>
       <c r="D28" s="4">
-        <v>124</v>
+        <v>145</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -1411,7 +1411,7 @@
         <v>1</v>
       </c>
       <c r="C29" s="4">
-        <v>500</v>
+        <v>585</v>
       </c>
     </row>
   </sheetData>
@@ -1794,22 +1794,22 @@
         <v>38</v>
       </c>
       <c r="B5">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C5">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="D5">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="E5">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="F5">
         <v>11</v>
       </c>
       <c r="G5">
-        <v>437</v>
+        <v>423</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -1817,22 +1817,22 @@
         <v>39</v>
       </c>
       <c r="B6">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C6">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="D6">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="E6">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="F6">
         <v>2</v>
       </c>
       <c r="G6">
-        <v>398</v>
+        <v>385</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -1840,13 +1840,13 @@
         <v>40</v>
       </c>
       <c r="B7">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C7">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D7">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E7">
         <v>37</v>
@@ -1855,7 +1855,7 @@
         <v>3</v>
       </c>
       <c r="G7">
-        <v>202</v>
+        <v>199</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -1863,22 +1863,22 @@
         <v>41</v>
       </c>
       <c r="B8">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C8">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D8">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E8">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F8">
         <v>0</v>
       </c>
       <c r="G8">
-        <v>97</v>
+        <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -1886,22 +1886,22 @@
         <v>42</v>
       </c>
       <c r="B9">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C9">
+        <v>24</v>
+      </c>
+      <c r="D9">
         <v>25</v>
       </c>
-      <c r="D9">
-        <v>27</v>
-      </c>
       <c r="E9">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F9">
         <v>0</v>
       </c>
       <c r="G9">
-        <v>75</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -1937,22 +1937,22 @@
         <v>38</v>
       </c>
       <c r="B13">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C13">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="D13">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="E13">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F13">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G13">
-        <v>461</v>
+        <v>446</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -1960,22 +1960,22 @@
         <v>39</v>
       </c>
       <c r="B14">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C14">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D14">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="E14">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F14">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G14">
-        <v>386</v>
+        <v>374</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -1989,16 +1989,16 @@
         <v>53</v>
       </c>
       <c r="D15">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E15">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F15">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G15">
-        <v>207</v>
+        <v>204</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -2006,22 +2006,22 @@
         <v>41</v>
       </c>
       <c r="B16">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C16">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D16">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E16">
+        <v>14</v>
+      </c>
+      <c r="F16">
         <v>15</v>
       </c>
-      <c r="F16">
-        <v>16</v>
-      </c>
       <c r="G16">
-        <v>84</v>
+        <v>77</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -2032,19 +2032,19 @@
         <v>6</v>
       </c>
       <c r="C17">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D17">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E17">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F17">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G17">
-        <v>61</v>
+        <v>56</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -2083,25 +2083,25 @@
         <v>38</v>
       </c>
       <c r="B21">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C21">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D21">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E21">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="F21">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="G21">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="H21">
-        <v>169</v>
+        <v>198</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -2109,25 +2109,25 @@
         <v>39</v>
       </c>
       <c r="B22">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C22">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D22">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E22">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="F22">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="G22">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="H22">
-        <v>146</v>
+        <v>171</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -2135,25 +2135,25 @@
         <v>41</v>
       </c>
       <c r="B23">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C23">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D23">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E23">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F23">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="G23">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="H23">
-        <v>89</v>
+        <v>104</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -2161,25 +2161,25 @@
         <v>42</v>
       </c>
       <c r="B24">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C24">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D24">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E24">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F24">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G24">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="H24">
-        <v>60</v>
+        <v>70</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -2187,25 +2187,25 @@
         <v>40</v>
       </c>
       <c r="B25">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C25">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D25">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E25">
         <v>5</v>
       </c>
       <c r="F25">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G25">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H25">
-        <v>36</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Explore Pants: ranking dashboard ajustado a tela comprada (sin déficit)
- Género×color ideal desde ranking ventas; cap por kg neto de tela
- KIDS 585, CAB/DAMA por ventas; tallas por curva dashboard
- Verificación tela: todos los colores con delta kg ≥ 0

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/EXPLORE_PANTS_Proyeccion_Produccion.xlsx
+++ b/EXPLORE_PANTS_Proyeccion_Produccion.xlsx
@@ -47,10 +47,10 @@
     <t>Pedido total archivo (Explore + Shorts): 1088 kg · split 65% / 35%</t>
   </si>
   <si>
-    <t>Color y talla: proporción del dashboard por género (ranking Colores/Tallas)</t>
-  </si>
-  <si>
-    <t>KIDS 550–620 und · CAB sin 3XL · verificación tela comprada</t>
+    <t>Color/talla: ranking dashboard por género, ajustado a tela comprada (sin déficit kg)</t>
+  </si>
+  <si>
+    <t>KIDS 550–620 und · CAB sin 3XL</t>
   </si>
   <si>
     <t>Consumo referencial: CAB 0.3 · DAMA 0.25 · KIDS 0.22 kg/und</t>
@@ -137,18 +137,18 @@
     <t>Negro</t>
   </si>
   <si>
+    <t>Gris Oscuro</t>
+  </si>
+  <si>
     <t>Kaki</t>
   </si>
   <si>
-    <t>Gris Oscuro</t>
+    <t>Azul Marino</t>
   </si>
   <si>
     <t>Verde Militar</t>
   </si>
   <si>
-    <t>Azul Marino</t>
-  </si>
-  <si>
     <t>EXPLORE PANTS — UNIDADES A PRODUCIR POR COLOR (TOTAL)</t>
   </si>
   <si>
@@ -329,7 +329,7 @@
     <t>1. TOTAL a producir: 2,908 und (80% pendiente, justificación Novaktex). La tela ya está comprada.</t>
   </si>
   <si>
-    <t>2. COLOR y TALLA: proporción del dashboard por género (misma curva que ranking Colores/Tallas).</t>
+    <t>2. COLOR y TALLA: ranking del dashboard por género; se ajusta iterativamente para no exceder kg de tela comprada.</t>
   </si>
   <si>
     <t>3. KIDS 550–620 und (meta 585); CAB/DAMA reparten el resto por ventas.</t>
@@ -338,7 +338,7 @@
     <t>4. CAB sin 3XL · KIDS sin talla 1 · Gris (ventas) → Gris Oscuro (producción).</t>
   </si>
   <si>
-    <t>5. Verificación tela: kg necesario vs kg comprado por color (consumo ref. CAB 0.3 · DAMA 0.25 · KIDS 0.22).</t>
+    <t>5. Verificación tela: kg necesario ≤ kg neto comprado por color (consumo ref. CAB 0.3 · DAMA 0.25 · KIDS 0.22).</t>
   </si>
   <si>
     <t>6. Demanda Jul–Dic (2,228 und) y escenarios mensuales del archivo de justificación.</t>
@@ -928,7 +928,7 @@
         <v>1185</v>
       </c>
       <c r="C30">
-        <v>1269</v>
+        <v>1270</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -939,7 +939,7 @@
         <v>1138</v>
       </c>
       <c r="C31">
-        <v>1218</v>
+        <v>1221</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -950,7 +950,7 @@
         <v>585</v>
       </c>
       <c r="C32">
-        <v>634</v>
+        <v>633</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -961,7 +961,7 @@
         <v>2908</v>
       </c>
       <c r="C33" s="5">
-        <v>3121</v>
+        <v>3124</v>
       </c>
     </row>
   </sheetData>
@@ -1006,10 +1006,10 @@
         <v>37</v>
       </c>
       <c r="B5" s="4">
-        <v>321</v>
+        <v>457</v>
       </c>
       <c r="C5" s="6">
-        <v>0.2708860759493671</v>
+        <v>0.3856540084388186</v>
       </c>
       <c r="D5" s="6">
         <v>0.272</v>
@@ -1020,13 +1020,13 @@
         <v>38</v>
       </c>
       <c r="B6" s="4">
-        <v>249</v>
+        <v>328</v>
       </c>
       <c r="C6" s="6">
-        <v>0.210126582278481</v>
+        <v>0.2767932489451477</v>
       </c>
       <c r="D6" s="6">
-        <v>0.21</v>
+        <v>0.196</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -1034,13 +1034,13 @@
         <v>39</v>
       </c>
       <c r="B7" s="4">
-        <v>233</v>
+        <v>218</v>
       </c>
       <c r="C7" s="6">
-        <v>0.1966244725738397</v>
+        <v>0.1839662447257384</v>
       </c>
       <c r="D7" s="6">
-        <v>0.196</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -1048,13 +1048,13 @@
         <v>40</v>
       </c>
       <c r="B8" s="4">
-        <v>192</v>
+        <v>103</v>
       </c>
       <c r="C8" s="6">
-        <v>0.1620253164556962</v>
+        <v>0.08691983122362869</v>
       </c>
       <c r="D8" s="6">
-        <v>0.162</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -1062,13 +1062,13 @@
         <v>41</v>
       </c>
       <c r="B9" s="4">
-        <v>190</v>
+        <v>79</v>
       </c>
       <c r="C9" s="6">
-        <v>0.160337552742616</v>
+        <v>0.06666666666666667</v>
       </c>
       <c r="D9" s="6">
-        <v>0.16</v>
+        <v>0.162</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -1106,10 +1106,10 @@
         <v>37</v>
       </c>
       <c r="B14" s="4">
-        <v>340</v>
+        <v>466</v>
       </c>
       <c r="C14" s="6">
-        <v>0.2987697715289983</v>
+        <v>0.4094903339191564</v>
       </c>
       <c r="D14" s="6">
         <v>0.298</v>
@@ -1120,13 +1120,13 @@
         <v>38</v>
       </c>
       <c r="B15" s="4">
-        <v>253</v>
+        <v>308</v>
       </c>
       <c r="C15" s="6">
-        <v>0.2223198594024605</v>
+        <v>0.2706502636203866</v>
       </c>
       <c r="D15" s="6">
-        <v>0.223</v>
+        <v>0.198</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -1134,24 +1134,24 @@
         <v>39</v>
       </c>
       <c r="B16" s="4">
-        <v>226</v>
+        <v>217</v>
       </c>
       <c r="C16" s="6">
-        <v>0.1985940246045694</v>
+        <v>0.1906854130052724</v>
       </c>
       <c r="D16" s="6">
-        <v>0.198</v>
+        <v>0.223</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B17" s="4">
-        <v>165</v>
+        <v>87</v>
       </c>
       <c r="C17" s="6">
-        <v>0.1449912126537786</v>
+        <v>0.07644991212653779</v>
       </c>
       <c r="D17" s="6">
         <v>0.145</v>
@@ -1159,13 +1159,13 @@
     </row>
     <row r="18" spans="1:4">
       <c r="A18" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B18" s="4">
-        <v>154</v>
+        <v>60</v>
       </c>
       <c r="C18" s="6">
-        <v>0.1353251318101933</v>
+        <v>0.05272407732864675</v>
       </c>
       <c r="D18" s="6">
         <v>0.136</v>
@@ -1203,69 +1203,69 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B23" s="4">
-        <v>166</v>
+        <v>214</v>
       </c>
       <c r="C23" s="6">
-        <v>0.2837606837606838</v>
+        <v>0.3658119658119658</v>
       </c>
       <c r="D23" s="6">
-        <v>0.284</v>
+        <v>0.225</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B24" s="4">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C24" s="6">
-        <v>0.2547008547008547</v>
+        <v>0.2495726495726496</v>
       </c>
       <c r="D24" s="6">
-        <v>0.253</v>
+        <v>0.154</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B25" s="4">
-        <v>132</v>
+        <v>104</v>
       </c>
       <c r="C25" s="6">
-        <v>0.2256410256410256</v>
+        <v>0.1777777777777778</v>
       </c>
       <c r="D25" s="6">
-        <v>0.225</v>
+        <v>0.284</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B26" s="4">
-        <v>90</v>
+        <v>71</v>
       </c>
       <c r="C26" s="6">
-        <v>0.1538461538461539</v>
+        <v>0.1213675213675214</v>
       </c>
       <c r="D26" s="6">
-        <v>0.154</v>
+        <v>0.253</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B27" s="4">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C27" s="6">
-        <v>0.08205128205128205</v>
+        <v>0.08547008547008547</v>
       </c>
       <c r="D27" s="6">
         <v>0.08400000000000001</v>
@@ -1319,10 +1319,10 @@
         <v>37</v>
       </c>
       <c r="B4" s="4">
-        <v>793</v>
+        <v>1137</v>
       </c>
       <c r="C4" s="6">
-        <v>0.2726960110041265</v>
+        <v>0.390990371389271</v>
       </c>
       <c r="D4" s="6">
         <v>0.3801652892561984</v>
@@ -1333,13 +1333,13 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B5" s="4">
-        <v>549</v>
+        <v>782</v>
       </c>
       <c r="C5" s="6">
-        <v>0.1887895460797799</v>
+        <v>0.2689133425034388</v>
       </c>
       <c r="D5" s="6">
         <v>0.3314967860422406</v>
@@ -1350,13 +1350,13 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B6" s="4">
-        <v>550</v>
+        <v>485</v>
       </c>
       <c r="C6" s="6">
-        <v>0.1891334250343879</v>
+        <v>0.1667812929848693</v>
       </c>
       <c r="D6" s="6">
         <v>0.1441689623507805</v>
@@ -1367,13 +1367,13 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B7" s="4">
-        <v>521</v>
+        <v>294</v>
       </c>
       <c r="C7" s="6">
-        <v>0.1791609353507565</v>
+        <v>0.1011004126547455</v>
       </c>
       <c r="D7" s="6">
         <v>0.08356290174471992</v>
@@ -1384,13 +1384,13 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B8" s="4">
-        <v>495</v>
+        <v>210</v>
       </c>
       <c r="C8" s="6">
-        <v>0.1702200825309491</v>
+        <v>0.07221458046767538</v>
       </c>
       <c r="D8" s="6">
         <v>0.06060606060606061</v>
@@ -1458,16 +1458,16 @@
         <v>52</v>
       </c>
       <c r="B5" s="6">
-        <v>0.1409282700421941</v>
+        <v>0.1451476793248945</v>
       </c>
       <c r="C5" s="6">
         <v>0.141</v>
       </c>
       <c r="D5" s="4">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="E5" s="4">
-        <v>180</v>
+        <v>185</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -1475,16 +1475,16 @@
         <v>53</v>
       </c>
       <c r="B6" s="6">
-        <v>0.3333333333333333</v>
+        <v>0.329957805907173</v>
       </c>
       <c r="C6" s="6">
         <v>0.334</v>
       </c>
       <c r="D6" s="4">
-        <v>395</v>
+        <v>391</v>
       </c>
       <c r="E6" s="4">
-        <v>421</v>
+        <v>418</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -1492,16 +1492,16 @@
         <v>54</v>
       </c>
       <c r="B7" s="6">
-        <v>0.3367088607594937</v>
+        <v>0.3341772151898734</v>
       </c>
       <c r="C7" s="6">
         <v>0.336</v>
       </c>
       <c r="D7" s="4">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="E7" s="4">
-        <v>425</v>
+        <v>423</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -1509,16 +1509,16 @@
         <v>55</v>
       </c>
       <c r="B8" s="6">
-        <v>0.1789029535864979</v>
+        <v>0.1763713080168776</v>
       </c>
       <c r="C8" s="6">
         <v>0.178</v>
       </c>
       <c r="D8" s="4">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="E8" s="4">
-        <v>228</v>
+        <v>224</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -1526,16 +1526,16 @@
         <v>56</v>
       </c>
       <c r="B9" s="6">
-        <v>0.01012658227848101</v>
+        <v>0.01434599156118144</v>
       </c>
       <c r="C9" s="6">
         <v>0.011</v>
       </c>
       <c r="D9" s="4">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E9" s="4">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -1579,16 +1579,16 @@
         <v>58</v>
       </c>
       <c r="B14" s="6">
-        <v>0.1230228471001757</v>
+        <v>0.1300527240773287</v>
       </c>
       <c r="C14" s="6">
         <v>0.122</v>
       </c>
       <c r="D14" s="4">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="E14" s="4">
-        <v>151</v>
+        <v>160</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -1596,16 +1596,16 @@
         <v>52</v>
       </c>
       <c r="B15" s="6">
-        <v>0.242530755711775</v>
+        <v>0.2478031634446397</v>
       </c>
       <c r="C15" s="6">
         <v>0.244</v>
       </c>
       <c r="D15" s="4">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="E15" s="4">
-        <v>295</v>
+        <v>301</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -1613,16 +1613,16 @@
         <v>53</v>
       </c>
       <c r="B16" s="6">
-        <v>0.304920913884007</v>
+        <v>0.3014059753954306</v>
       </c>
       <c r="C16" s="6">
         <v>0.305</v>
       </c>
       <c r="D16" s="4">
-        <v>347</v>
+        <v>343</v>
       </c>
       <c r="E16" s="4">
-        <v>370</v>
+        <v>367</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -1630,16 +1630,16 @@
         <v>54</v>
       </c>
       <c r="B17" s="6">
-        <v>0.1766256590509666</v>
+        <v>0.1704745166959578</v>
       </c>
       <c r="C17" s="6">
         <v>0.176</v>
       </c>
       <c r="D17" s="4">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="E17" s="4">
-        <v>215</v>
+        <v>208</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -1647,16 +1647,16 @@
         <v>55</v>
       </c>
       <c r="B18" s="6">
-        <v>0.1520210896309315</v>
+        <v>0.1493848857644991</v>
       </c>
       <c r="C18" s="6">
         <v>0.153</v>
       </c>
       <c r="D18" s="4">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="E18" s="4">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -1717,16 +1717,16 @@
         <v>60</v>
       </c>
       <c r="B24" s="6">
-        <v>0.0905982905982906</v>
+        <v>0.105982905982906</v>
       </c>
       <c r="C24" s="6">
         <v>0.09300000000000001</v>
       </c>
       <c r="D24" s="4">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="E24" s="4">
-        <v>59</v>
+        <v>68</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -1734,16 +1734,16 @@
         <v>61</v>
       </c>
       <c r="B25" s="6">
-        <v>0.1299145299145299</v>
+        <v>0.1316239316239316</v>
       </c>
       <c r="C25" s="6">
         <v>0.131</v>
       </c>
       <c r="D25" s="4">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E25" s="4">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -1751,16 +1751,16 @@
         <v>62</v>
       </c>
       <c r="B26" s="6">
-        <v>0.1145299145299145</v>
+        <v>0.1076923076923077</v>
       </c>
       <c r="C26" s="6">
         <v>0.115</v>
       </c>
       <c r="D26" s="4">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="E26" s="4">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -1768,16 +1768,16 @@
         <v>63</v>
       </c>
       <c r="B27" s="6">
-        <v>0.2</v>
+        <v>0.2034188034188034</v>
       </c>
       <c r="C27" s="6">
         <v>0.198</v>
       </c>
       <c r="D27" s="4">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E27" s="4">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -1785,16 +1785,16 @@
         <v>64</v>
       </c>
       <c r="B28" s="6">
-        <v>0.2170940170940171</v>
+        <v>0.2205128205128205</v>
       </c>
       <c r="C28" s="6">
         <v>0.215</v>
       </c>
       <c r="D28" s="4">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E28" s="4">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -1802,16 +1802,16 @@
         <v>65</v>
       </c>
       <c r="B29" s="6">
-        <v>0.2478632478632479</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="C29" s="6">
         <v>0.248</v>
       </c>
       <c r="D29" s="4">
+        <v>135</v>
+      </c>
+      <c r="E29" s="4">
         <v>145</v>
-      </c>
-      <c r="E29" s="4">
-        <v>156</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -1876,114 +1876,114 @@
         <v>37</v>
       </c>
       <c r="B6" s="4">
-        <v>793</v>
+        <v>1137</v>
       </c>
       <c r="C6" s="6">
-        <v>0.273</v>
+        <v>0.391</v>
       </c>
       <c r="D6" s="6">
         <v>0.38</v>
       </c>
       <c r="E6" s="8">
-        <v>210.3</v>
+        <v>300.7</v>
       </c>
       <c r="F6" s="8">
         <v>345</v>
       </c>
       <c r="G6" s="8">
-        <v>134.7</v>
+        <v>44.3</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B7" s="4">
-        <v>549</v>
+        <v>782</v>
       </c>
       <c r="C7" s="6">
-        <v>0.189</v>
+        <v>0.269</v>
       </c>
       <c r="D7" s="6">
         <v>0.331</v>
       </c>
       <c r="E7" s="8">
-        <v>146.2</v>
+        <v>207.5</v>
       </c>
       <c r="F7" s="8">
         <v>300.8</v>
       </c>
       <c r="G7" s="8">
-        <v>154.6</v>
+        <v>93.3</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B8" s="4">
-        <v>550</v>
+        <v>485</v>
       </c>
       <c r="C8" s="6">
-        <v>0.189</v>
+        <v>0.167</v>
       </c>
       <c r="D8" s="6">
         <v>0.144</v>
       </c>
       <c r="E8" s="8">
-        <v>148.5</v>
+        <v>130.6</v>
       </c>
       <c r="F8" s="8">
         <v>130.8</v>
       </c>
       <c r="G8" s="8">
-        <v>-17.7</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B9" s="4">
-        <v>521</v>
+        <v>294</v>
       </c>
       <c r="C9" s="6">
-        <v>0.179</v>
+        <v>0.101</v>
       </c>
       <c r="D9" s="6">
         <v>0.08400000000000001</v>
       </c>
       <c r="E9" s="8">
-        <v>134.8</v>
+        <v>75.5</v>
       </c>
       <c r="F9" s="8">
         <v>75.8</v>
       </c>
       <c r="G9" s="8">
-        <v>-58.9</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B10" s="4">
-        <v>495</v>
+        <v>210</v>
       </c>
       <c r="C10" s="6">
-        <v>0.17</v>
+        <v>0.07200000000000001</v>
       </c>
       <c r="D10" s="6">
         <v>0.061</v>
       </c>
       <c r="E10" s="8">
-        <v>128.9</v>
+        <v>54.3</v>
       </c>
       <c r="F10" s="8">
         <v>55</v>
       </c>
       <c r="G10" s="8">
-        <v>-73.90000000000001</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -1994,13 +1994,13 @@
         <v>2908</v>
       </c>
       <c r="E11" s="8">
-        <v>768.7</v>
+        <v>768.6</v>
       </c>
       <c r="F11" s="8">
         <v>907.4</v>
       </c>
       <c r="G11" s="8">
-        <v>138.7</v>
+        <v>138.8</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -2247,22 +2247,22 @@
         <v>37</v>
       </c>
       <c r="B5">
-        <v>42</v>
+        <v>60</v>
       </c>
       <c r="C5">
-        <v>106</v>
+        <v>151</v>
       </c>
       <c r="D5">
-        <v>108</v>
+        <v>153</v>
       </c>
       <c r="E5">
-        <v>57</v>
+        <v>81</v>
       </c>
       <c r="F5">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G5">
-        <v>321</v>
+        <v>457</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -2270,22 +2270,22 @@
         <v>38</v>
       </c>
       <c r="B6">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="C6">
-        <v>83</v>
+        <v>105</v>
       </c>
       <c r="D6">
-        <v>77</v>
+        <v>113</v>
       </c>
       <c r="E6">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="F6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G6">
-        <v>249</v>
+        <v>328</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -2293,22 +2293,22 @@
         <v>39</v>
       </c>
       <c r="B7">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C7">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D7">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="E7">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G7">
-        <v>233</v>
+        <v>218</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -2316,22 +2316,22 @@
         <v>40</v>
       </c>
       <c r="B8">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="C8">
-        <v>65</v>
+        <v>36</v>
       </c>
       <c r="D8">
-        <v>69</v>
+        <v>35</v>
       </c>
       <c r="E8">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="F8">
         <v>0</v>
       </c>
       <c r="G8">
-        <v>192</v>
+        <v>103</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -2339,22 +2339,22 @@
         <v>41</v>
       </c>
       <c r="B9">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="C9">
-        <v>67</v>
+        <v>27</v>
       </c>
       <c r="D9">
-        <v>65</v>
+        <v>28</v>
       </c>
       <c r="E9">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="F9">
         <v>0</v>
       </c>
       <c r="G9">
-        <v>190</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -2393,25 +2393,25 @@
         <v>37</v>
       </c>
       <c r="B13">
-        <v>54</v>
+        <v>73</v>
       </c>
       <c r="C13">
-        <v>84</v>
+        <v>116</v>
       </c>
       <c r="D13">
-        <v>101</v>
+        <v>138</v>
       </c>
       <c r="E13">
-        <v>51</v>
+        <v>70</v>
       </c>
       <c r="F13">
-        <v>50</v>
+        <v>69</v>
       </c>
       <c r="G13">
         <v>0</v>
       </c>
       <c r="H13">
-        <v>340</v>
+        <v>466</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -2419,25 +2419,25 @@
         <v>38</v>
       </c>
       <c r="B14">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="C14">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="D14">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="E14">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="F14">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="G14">
         <v>0</v>
       </c>
       <c r="H14">
-        <v>253</v>
+        <v>308</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -2445,77 +2445,77 @@
         <v>39</v>
       </c>
       <c r="B15">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C15">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D15">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E15">
         <v>41</v>
       </c>
       <c r="F15">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="G15">
         <v>0</v>
       </c>
       <c r="H15">
-        <v>226</v>
+        <v>217</v>
       </c>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B16">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="C16">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="D16">
-        <v>57</v>
+        <v>30</v>
       </c>
       <c r="E16">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="F16">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="G16">
         <v>1</v>
       </c>
       <c r="H16">
-        <v>165</v>
+        <v>87</v>
       </c>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B17">
+        <v>7</v>
+      </c>
+      <c r="C17">
+        <v>15</v>
+      </c>
+      <c r="D17">
         <v>17</v>
       </c>
-      <c r="C17">
-        <v>38</v>
-      </c>
-      <c r="D17">
-        <v>44</v>
-      </c>
       <c r="E17">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="F17">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="G17">
         <v>0</v>
       </c>
       <c r="H17">
-        <v>154</v>
+        <v>60</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -2551,111 +2551,111 @@
     </row>
     <row r="21" spans="1:8">
       <c r="A21" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B21">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="C21">
+        <v>28</v>
+      </c>
+      <c r="D21">
         <v>23</v>
       </c>
-      <c r="D21">
-        <v>16</v>
-      </c>
       <c r="E21">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="F21">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="G21">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="H21">
-        <v>166</v>
+        <v>214</v>
       </c>
     </row>
     <row r="22" spans="1:8">
       <c r="A22" t="s">
+        <v>38</v>
+      </c>
+      <c r="B22">
+        <v>15</v>
+      </c>
+      <c r="C22">
+        <v>18</v>
+      </c>
+      <c r="D22">
+        <v>12</v>
+      </c>
+      <c r="E22">
         <v>40</v>
       </c>
-      <c r="B22">
-        <v>10</v>
-      </c>
-      <c r="C22">
-        <v>16</v>
-      </c>
-      <c r="D22">
-        <v>23</v>
-      </c>
-      <c r="E22">
+      <c r="F22">
+        <v>31</v>
+      </c>
+      <c r="G22">
         <v>30</v>
       </c>
-      <c r="F22">
-        <v>30</v>
-      </c>
-      <c r="G22">
-        <v>40</v>
-      </c>
       <c r="H22">
-        <v>149</v>
+        <v>146</v>
       </c>
     </row>
     <row r="23" spans="1:8">
       <c r="A23" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B23">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C23">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D23">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E23">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F23">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="G23">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="H23">
-        <v>132</v>
+        <v>104</v>
       </c>
     </row>
     <row r="24" spans="1:8">
       <c r="A24" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B24">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C24">
+        <v>8</v>
+      </c>
+      <c r="D24">
         <v>11</v>
       </c>
-      <c r="D24">
-        <v>7</v>
-      </c>
       <c r="E24">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="F24">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="G24">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H24">
-        <v>90</v>
+        <v>71</v>
       </c>
     </row>
     <row r="25" spans="1:8">
       <c r="A25" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B25">
         <v>4</v>
@@ -2670,13 +2670,13 @@
         <v>6</v>
       </c>
       <c r="F25">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G25">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H25">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>